<commit_message>
Tipo de equipo: criterios del Anexo I.2 según el tipo
El Anexo I.2 del RD 1215/1997 solo aplica a determinados tipos de equipo
(móviles, elevación de cargas), pero el modelo no podía expresarlo. Se añade
TipoEquipo, Equipo.tipos y GrupoCriterio.tipos_aplicables: un grupo sin tipos
aplica a todos los equipos; con tipos, solo a esos. Relación M2M porque un
equipo puede ser de varios tipos a la vez (la carretilla elevadora es equipo
móvil y de elevación).

Se amplía el inventario de ejemplo con puente grúa, carretilla elevadora y
llave dinamométrica, de modo que el caso de estudio cubra también el
Anexo I.2 y el numeral 19 del Anexo I.1.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ejemplos_importacion/equipos_ok.xlsx
+++ b/docs/ejemplos_importacion/equipos_ok.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -549,10 +549,6 @@
           <t>Compresor</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -612,6 +608,81 @@
         <is>
           <t>Línea 3</t>
         </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EQ-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Puente grúa</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ACME PG50</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SN-1007</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EQ-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Carretilla elevadora</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ACME CE25</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SN-1008</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EQ-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Llave dinamométrica</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Stahlwille 730</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SN-1009</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>2023</v>
       </c>
     </row>
   </sheetData>

</xml_diff>